<commit_message>
feat: MaxDiff module v11.0 upgrade
Add four analytical innovations (TURF portfolio optimization, preference
shares, anchored MaxDiff, item discrimination), HTML report pipeline,
interactive simulator, demo showcase, and testthat test suite. Update
config template with new settings and fix validation edge cases.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/maxdiff/templates/maxdiff_config_template.xlsx
+++ b/modules/maxdiff/templates/maxdiff_config_template.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="294">
   <si>
     <t xml:space="preserve">Topic</t>
   </si>
@@ -251,10 +251,34 @@
     <t xml:space="preserve">12345, 42, 98765</t>
   </si>
   <si>
+    <t xml:space="preserve">Brand_Colour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#1e3a5f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primary brand colour for HTML report and simulator (hex format)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#1e3a5f, #2c3e50, #003366</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accent_Colour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#2aa198</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secondary accent colour for HTML report (hex format)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#2aa198, #e67e22, #27ae60</t>
+  </si>
+  <si>
     <t xml:space="preserve">Module_Version</t>
   </si>
   <si>
-    <t xml:space="preserve">v10.0</t>
+    <t xml:space="preserve">v11.0</t>
   </si>
   <si>
     <t xml:space="preserve">Module version (for tracking)</t>
@@ -596,6 +620,15 @@
     <t xml:space="preserve">Worst_Value_Type</t>
   </si>
   <si>
+    <t xml:space="preserve">Anchor_Variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Column containing anchor/must-have selections (comma-separated Item_IDs or blank)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MustHave_Items, Anchor_Q (e.g. 'ITEM_01,ITEM_03,ITEM_05')</t>
+  </si>
+  <si>
     <t xml:space="preserve">Note</t>
   </si>
   <si>
@@ -725,7 +758,88 @@
     <t xml:space="preserve">Generate_Charts</t>
   </si>
   <si>
-    <t xml:space="preserve">Generate visualization charts</t>
+    <t xml:space="preserve">Generate PNG/PDF visualization charts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generate_HTML_Report</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generate interactive HTML report with SVG charts and tabbed layout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YES or NO (produces self-contained .html file)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generate_Simulator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generate interactive HTML simulator (head-to-head, portfolio builder)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YES or NO (requires HB or logit results)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generate_TURF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run TURF (Total Unduplicated Reach &amp; Frequency) portfolio optimization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YES or NO (requires individual-level utilities from HB)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TURF_Max_Items</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximum portfolio size for TURF analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 to n_items (default: min(10, n_items))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TURF_Threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Method for classifying items as appealing in TURF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTO | TOP_3 | ABOVE_MEAN | ABOVE_ZERO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Has_Anchor_Question</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whether the survey includes an anchor/must-have question</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anchor_Threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proportion threshold for classifying items as must-have (0.0-1.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0-1.0 (items with anchor rate above this = must-have)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Score_Display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOTH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How to display preference scores in reports</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UTILITY | PREFERENCE_SHARE | BOTH</t>
   </si>
   <si>
     <t xml:space="preserve">Utility_Scale</t>
@@ -1749,7 +1863,41 @@
         <v>79</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>78</v>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1774,36 +1922,36 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="D2" s="5" t="n">
         <v>1</v>
@@ -1820,13 +1968,13 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="D3" s="5" t="n">
         <v>1</v>
@@ -1843,13 +1991,13 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>1</v>
@@ -1866,13 +2014,13 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>1</v>
@@ -1889,13 +2037,13 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>1</v>
@@ -1912,13 +2060,13 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>1</v>
@@ -1935,13 +2083,13 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>1</v>
@@ -1958,13 +2106,13 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>1</v>
@@ -1981,13 +2129,13 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>1</v>
@@ -2004,13 +2152,13 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>1</v>
@@ -2027,7 +2175,7 @@
     </row>
     <row r="14">
       <c r="A14" s="6" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>36</v>
@@ -2038,79 +2186,79 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>56</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>56</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>56</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>56</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>56</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -2134,7 +2282,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>35</v>
@@ -2146,55 +2294,55 @@
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>40</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>40</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>60</v>
@@ -2203,38 +2351,38 @@
         <v>56</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>56</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>40</v>
@@ -2243,38 +2391,38 @@
         <v>56</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>56</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>40</v>
@@ -2283,10 +2431,10 @@
         <v>56</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>40</v>
@@ -2294,7 +2442,7 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>40</v>
@@ -2303,10 +2451,10 @@
         <v>56</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>40</v>
@@ -2314,7 +2462,7 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>40</v>
@@ -2323,10 +2471,10 @@
         <v>56</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>40</v>
@@ -2334,42 +2482,42 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>56</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>56</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -2392,7 +2540,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>35</v>
@@ -2404,134 +2552,151 @@
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>40</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>40</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>40</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>56</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>40</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>40</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>190</v>
+        <v>198</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>196</v>
+        <v>207</v>
       </c>
     </row>
     <row r="15">
@@ -2541,17 +2706,17 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>198</v>
+        <v>209</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -2575,33 +2740,33 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>60</v>
@@ -2615,16 +2780,16 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>206</v>
+        <v>217</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>207</v>
+        <v>218</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>1</v>
@@ -2635,13 +2800,13 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>209</v>
+        <v>220</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>60</v>
@@ -2655,16 +2820,16 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>210</v>
+        <v>221</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>207</v>
+        <v>218</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>1</v>
@@ -2675,16 +2840,16 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>211</v>
+        <v>222</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>1</v>
@@ -2695,16 +2860,16 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>213</v>
+        <v>224</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>213</v>
+        <v>224</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>1</v>
@@ -2715,16 +2880,16 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>1</v>
@@ -2735,16 +2900,16 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="E9" s="5" t="n">
         <v>1</v>
@@ -2755,16 +2920,16 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>216</v>
+        <v>227</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>216</v>
+        <v>227</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>1</v>
@@ -2775,7 +2940,7 @@
     </row>
     <row r="13">
       <c r="A13" s="6" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>36</v>
@@ -2786,68 +2951,68 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>56</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>56</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -2878,175 +3043,287 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>225</v>
+        <v>236</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>226</v>
+        <v>237</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>227</v>
+        <v>238</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>56</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>230</v>
+        <v>241</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>231</v>
+        <v>242</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
-        <v>232</v>
+        <v>243</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
-        <v>234</v>
+        <v>245</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>235</v>
+        <v>246</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>237</v>
+        <v>40</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>145</v>
+        <v>252</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="s">
-        <v>242</v>
+        <v>253</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>243</v>
+        <v>254</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>145</v>
+        <v>255</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>253</v>
+        <v>56</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>254</v>
+        <v>265</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>255</v>
+        <v>153</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>293</v>
       </c>
     </row>
   </sheetData>

</xml_diff>